<commit_message>
Final - Spring 2025
</commit_message>
<xml_diff>
--- a/backend/data/mid1.xlsx
+++ b/backend/data/mid1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\PycharmProjects\pythonProject\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Date Sheet\backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{24B8D9A6-0749-414F-99F1-FD9DC549259F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{02CCEDC3-BA84-415B-9DA5-C2B4C6E42372}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B9985004-6A28-4E7A-8E55-DEE1FA60F161}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7FFC8B02-EDD0-430E-BBF0-A2BB718037AE}"/>
   </bookViews>
   <sheets>
     <sheet name="Complete" sheetId="5" r:id="rId1"/>
@@ -20,7 +20,9 @@
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
         <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
@@ -31,10 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="754" uniqueCount="495">
-  <si>
-    <t>Spring 2025 Semester</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="762" uniqueCount="498">
   <si>
     <t>Day</t>
   </si>
@@ -399,9 +398,6 @@
     <t>CS4001</t>
   </si>
   <si>
-    <t>Professional Practices in IT</t>
-  </si>
-  <si>
     <t>EE5050</t>
   </si>
   <si>
@@ -516,9 +512,6 @@
     <t>CL1002</t>
   </si>
   <si>
-    <t>Programming Fundamentals - Lab</t>
-  </si>
-  <si>
     <t>SL3003</t>
   </si>
   <si>
@@ -528,9 +521,6 @@
     <t>MG2010</t>
   </si>
   <si>
-    <t>Business Communication</t>
-  </si>
-  <si>
     <t>SS5004</t>
   </si>
   <si>
@@ -540,9 +530,6 @@
     <t>CV5057</t>
   </si>
   <si>
-    <t>Advanced Soil Mechanics</t>
-  </si>
-  <si>
     <t>MG1002</t>
   </si>
   <si>
@@ -852,9 +839,6 @@
     <t>CS4054</t>
   </si>
   <si>
-    <t>Bioinformatics</t>
-  </si>
-  <si>
     <t>CV5055</t>
   </si>
   <si>
@@ -1044,18 +1028,12 @@
     <t>MG5024</t>
   </si>
   <si>
-    <t>Cases in Management</t>
-  </si>
-  <si>
     <t>MT2005</t>
   </si>
   <si>
     <t>CV5066</t>
   </si>
   <si>
-    <t>Earthquake Engineering</t>
-  </si>
-  <si>
     <t>DS3002</t>
   </si>
   <si>
@@ -1071,15 +1049,9 @@
     <t>CV2009</t>
   </si>
   <si>
-    <t>Civil Engineering Graphics &amp;amp; Construction</t>
-  </si>
-  <si>
     <t>NS1001</t>
   </si>
   <si>
-    <t>Applied Physics</t>
-  </si>
-  <si>
     <t>DL3002</t>
   </si>
   <si>
@@ -1089,9 +1061,6 @@
     <t>MT5002</t>
   </si>
   <si>
-    <t>Advanced Integral Equations</t>
-  </si>
-  <si>
     <t>EE6011</t>
   </si>
   <si>
@@ -1101,9 +1070,6 @@
     <t>MG3002</t>
   </si>
   <si>
-    <t>Business Law</t>
-  </si>
-  <si>
     <t>BA4001</t>
   </si>
   <si>
@@ -1179,9 +1145,6 @@
     <t>DL2004</t>
   </si>
   <si>
-    <t>Fundamental of Big Data Analytics - Lab</t>
-  </si>
-  <si>
     <t>MG1009</t>
   </si>
   <si>
@@ -1203,9 +1166,6 @@
     <t>SS2008</t>
   </si>
   <si>
-    <t>Business Communication–I</t>
-  </si>
-  <si>
     <t>MG4013</t>
   </si>
   <si>
@@ -1515,14 +1475,88 @@
     <t>Electro-Mechanical Systems</t>
   </si>
   <si>
+    <t>Marketing Management (FSC)</t>
+  </si>
+  <si>
+    <t>Marketing Management (FSM)</t>
+  </si>
+  <si>
     <t>COMPLETE DATE SHEET FOR FINAL EXAMS</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Spring 2025 Semester              </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="14"/>
+        <color indexed="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>STU</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color indexed="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>-1.4</t>
+    </r>
+  </si>
+  <si>
+    <t>Professional Practices in IT (2:30-5:30PM)</t>
+  </si>
+  <si>
+    <t>Advanced Soil Mechanics (2:30-5:30PM)</t>
+  </si>
+  <si>
+    <t>Business Communication–I (2:30-5:30PM)</t>
+  </si>
+  <si>
+    <t>Business Communication (2:30-5:30PM)</t>
+  </si>
+  <si>
+    <t>Critical Thinking (2:30-5:30PM)</t>
+  </si>
+  <si>
+    <t>Programming Fundamentals - Lab  (2:30-5:30PM)</t>
+  </si>
+  <si>
+    <t>Civil Engineering Graphics &amp;amp; Construction (2:30-5:30PM)</t>
+  </si>
+  <si>
+    <t>Applied Physics (2:30-5:30PM)</t>
+  </si>
+  <si>
+    <t>Fundamental of Big Data Analytics - Lab (2:30-5:30PM)</t>
+  </si>
+  <si>
+    <t>Advanced Integral Equations (2:30-5:30PM)</t>
+  </si>
+  <si>
+    <t>Earthquake Engineering (2:30-5:30PM)</t>
+  </si>
+  <si>
+    <t>Business Law (2:30-5:30PM)</t>
+  </si>
+  <si>
+    <t>Bioinformatics (2:30-5:30PM)</t>
+  </si>
+  <si>
+    <t>Cases in Management (2:30-5:30PM)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -1536,6 +1570,7 @@
       <sz val="14"/>
       <color indexed="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -1543,29 +1578,54 @@
       <sz val="14"/>
       <color indexed="23"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color indexed="8"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color indexed="8"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <i/>
       <sz val="14"/>
-      <color theme="8" tint="-0.499984740745262"/>
+      <color indexed="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color indexed="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="14"/>
+      <color theme="4" tint="-0.499984740745262"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1580,6 +1640,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="3" tint="0.89999084444715716"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1620,7 +1692,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1632,13 +1704,19 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1974,8 +2052,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDCF6D9D-4F34-4ECF-9CFB-C4BC653607DD}">
-  <dimension ref="A1:I150"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A8ADFA4-A4DA-47B1-979F-5A9D05B741C4}">
+  <dimension ref="A1:I153"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.6640625" bestFit="1" customWidth="1"/>
@@ -1987,381 +2065,385 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
-        <v>494</v>
-      </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="5"/>
-      <c r="H1" s="5"/>
-      <c r="I1" s="6"/>
+      <c r="A1" s="10" t="s">
+        <v>482</v>
+      </c>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+      <c r="I1" s="7"/>
     </row>
     <row r="2" spans="1:9" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A2" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="6"/>
+      <c r="A2" s="11" t="s">
+        <v>483</v>
+      </c>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="11"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8"/>
+      <c r="I2" s="7"/>
     </row>
     <row r="3" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="C3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="D3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>4</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>7</v>
-      </c>
       <c r="C4" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>42</v>
-      </c>
       <c r="E4" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F4" s="4" t="s">
         <v>49</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>7</v>
-      </c>
       <c r="C5" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="E5" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="F5" s="4" t="s">
         <v>51</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>7</v>
-      </c>
       <c r="C6" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>32</v>
-      </c>
       <c r="E6" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>47</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>7</v>
-      </c>
       <c r="C7" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="D7" s="2" t="s">
-        <v>34</v>
-      </c>
       <c r="E7" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="F7" s="2" t="s">
         <v>45</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>7</v>
-      </c>
       <c r="C8" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="D8" s="2" t="s">
-        <v>36</v>
-      </c>
       <c r="E8" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F8" s="2" t="s">
         <v>61</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>7</v>
-      </c>
       <c r="C9" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D9" s="2" t="s">
-        <v>30</v>
-      </c>
       <c r="E9" s="2" t="s">
-        <v>53</v>
+        <v>403</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>54</v>
+        <v>404</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>7</v>
-      </c>
       <c r="C10" s="2" t="s">
-        <v>39</v>
+        <v>284</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>40</v>
+        <v>285</v>
       </c>
       <c r="E10" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F10" s="2" t="s">
         <v>55</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B11" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
+      <c r="C11" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>184</v>
+      </c>
       <c r="E11" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="F11" s="2" t="s">
         <v>57</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B12" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
+      <c r="C12" s="2" t="s">
+        <v>445</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>33</v>
+      </c>
       <c r="E12" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="F12" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="F12" s="2" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
+    </row>
+    <row r="13" spans="1:9" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>172</v>
+      </c>
     </row>
     <row r="14" spans="1:9" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>66</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
       <c r="E14" s="2" t="s">
-        <v>75</v>
+        <v>424</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="E15" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="F15" s="4" t="s">
-        <v>78</v>
-      </c>
+        <v>425</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A15" s="3"/>
+      <c r="B15" s="3"/>
+      <c r="C15" s="3"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
     </row>
     <row r="16" spans="1:9" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B16" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>409</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>410</v>
+      <c r="C16" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>480</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B17" s="2" t="s">
-        <v>9</v>
-      </c>
       <c r="C17" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>82</v>
+        <v>71</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B18" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B18" s="2" t="s">
-        <v>9</v>
-      </c>
       <c r="C18" s="2" t="s">
-        <v>73</v>
+        <v>395</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>74</v>
+        <v>396</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B19" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B19" s="2" t="s">
-        <v>9</v>
-      </c>
       <c r="C19" s="2" t="s">
-        <v>170</v>
+        <v>66</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>171</v>
+        <v>67</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B20" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B20" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
+      <c r="C20" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>115</v>
+      </c>
       <c r="E20" s="2" t="s">
-        <v>87</v>
+        <v>68</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>88</v>
+        <v>69</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B21" s="2" t="s">
         <v>8</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>9</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" s="2"/>
       <c r="E21" s="2" t="s">
-        <v>69</v>
+        <v>84</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>70</v>
+        <v>85</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
@@ -2374,2331 +2456,2367 @@
     </row>
     <row r="23" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B23" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B23" s="2" t="s">
-        <v>11</v>
-      </c>
       <c r="C23" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="D23" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="D23" s="2" t="s">
-        <v>90</v>
-      </c>
       <c r="E23" s="2" t="s">
-        <v>101</v>
+        <v>210</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>102</v>
+        <v>211</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B24" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B24" s="2" t="s">
-        <v>11</v>
-      </c>
       <c r="C24" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="D24" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="D24" s="2" t="s">
-        <v>92</v>
-      </c>
       <c r="E24" s="2" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B25" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B25" s="2" t="s">
-        <v>11</v>
-      </c>
       <c r="C25" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="D25" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="D25" s="2" t="s">
-        <v>98</v>
-      </c>
       <c r="E25" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="F25" s="4" t="s">
         <v>105</v>
-      </c>
-      <c r="F25" s="4" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B26" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B26" s="2" t="s">
-        <v>11</v>
-      </c>
       <c r="C26" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="D26" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="D26" s="2" t="s">
-        <v>94</v>
-      </c>
       <c r="E26" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="F26" s="2" t="s">
         <v>107</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B27" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B27" s="2" t="s">
-        <v>11</v>
-      </c>
       <c r="C27" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="D27" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="D27" s="2" t="s">
-        <v>100</v>
-      </c>
       <c r="E27" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="F27" s="2" t="s">
         <v>109</v>
-      </c>
-      <c r="F27" s="2" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B28" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B28" s="2" t="s">
-        <v>11</v>
-      </c>
       <c r="C28" s="2" t="s">
-        <v>442</v>
+        <v>428</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>443</v>
+        <v>429</v>
       </c>
       <c r="E28" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="F28" s="2" t="s">
         <v>111</v>
-      </c>
-      <c r="F28" s="2" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B29" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B29" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C29" s="2"/>
-      <c r="D29" s="2"/>
+      <c r="C29" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>39</v>
+      </c>
       <c r="E29" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="F29" s="2" t="s">
         <v>113</v>
-      </c>
-      <c r="F29" s="2" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B30" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B30" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
+      <c r="C30" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>73</v>
+      </c>
       <c r="E30" s="2" t="s">
-        <v>215</v>
+        <v>420</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31" s="3"/>
-      <c r="B31" s="3"/>
-      <c r="C31" s="3"/>
-      <c r="D31" s="3"/>
-      <c r="E31" s="3"/>
-      <c r="F31" s="3"/>
-    </row>
-    <row r="32" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="E32" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="F32" s="2" t="s">
-        <v>104</v>
-      </c>
+        <v>421</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C31" s="2"/>
+      <c r="D31" s="2"/>
+      <c r="E31" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A32" s="3"/>
+      <c r="B32" s="3"/>
+      <c r="C32" s="3"/>
+      <c r="D32" s="3"/>
+      <c r="E32" s="3"/>
+      <c r="F32" s="3"/>
     </row>
     <row r="33" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B33" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B33" s="2" t="s">
-        <v>13</v>
-      </c>
       <c r="C33" s="2" t="s">
-        <v>117</v>
+        <v>42</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>118</v>
+        <v>43</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>141</v>
+        <v>102</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>142</v>
+        <v>103</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B34" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B34" s="2" t="s">
-        <v>13</v>
-      </c>
       <c r="C34" s="2" t="s">
-        <v>119</v>
+        <v>133</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>120</v>
+        <v>134</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B35" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B35" s="2" t="s">
-        <v>13</v>
-      </c>
       <c r="C35" s="2" t="s">
-        <v>133</v>
+        <v>118</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="E35" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="F35" s="4" t="s">
-        <v>146</v>
+        <v>119</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="36" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B36" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B36" s="2" t="s">
-        <v>13</v>
-      </c>
       <c r="C36" s="2" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="E36" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="F36" s="2" t="s">
-        <v>148</v>
+        <v>132</v>
+      </c>
+      <c r="E36" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="F36" s="4" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="37" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B37" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B37" s="2" t="s">
-        <v>13</v>
-      </c>
       <c r="C37" s="2" t="s">
-        <v>153</v>
+        <v>121</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="E37" s="4" t="s">
-        <v>162</v>
-      </c>
-      <c r="F37" s="4" t="s">
-        <v>163</v>
+        <v>122</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="38" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B38" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B38" s="2" t="s">
-        <v>13</v>
-      </c>
       <c r="C38" s="2" t="s">
-        <v>127</v>
+        <v>151</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="E38" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="F38" s="2" t="s">
-        <v>132</v>
+        <v>152</v>
+      </c>
+      <c r="E38" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="F38" s="4" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="39" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B39" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B39" s="2" t="s">
-        <v>13</v>
-      </c>
       <c r="C39" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="E39" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="D39" s="2" t="s">
+      <c r="F39" s="2" t="s">
         <v>130</v>
-      </c>
-      <c r="E39" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="F39" s="2" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="40" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B40" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B40" s="2" t="s">
-        <v>13</v>
-      </c>
       <c r="C40" s="2" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="E40" s="2"/>
-      <c r="F40" s="2"/>
+        <v>128</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="41" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B41" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B41" s="2" t="s">
-        <v>13</v>
-      </c>
       <c r="C41" s="2" t="s">
-        <v>43</v>
+        <v>123</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="E41" s="2"/>
-      <c r="F41" s="2"/>
+        <v>124</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="42" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B42" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B42" s="2" t="s">
-        <v>13</v>
-      </c>
       <c r="C42" s="2" t="s">
-        <v>135</v>
+        <v>147</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="E42" s="2"/>
-      <c r="F42" s="2"/>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A43" s="3"/>
-      <c r="B43" s="3"/>
-      <c r="C43" s="3"/>
-      <c r="D43" s="3"/>
-      <c r="E43" s="3"/>
-      <c r="F43" s="3"/>
-    </row>
-    <row r="44" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B44" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C44" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="D44" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="E44" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="F44" s="4" t="s">
-        <v>161</v>
-      </c>
+        <v>148</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="E43" s="2"/>
+      <c r="F43" s="2"/>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A44" s="3"/>
+      <c r="B44" s="3"/>
+      <c r="C44" s="3"/>
+      <c r="D44" s="3"/>
+      <c r="E44" s="3"/>
+      <c r="F44" s="3"/>
     </row>
     <row r="45" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B45" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B45" s="2" t="s">
-        <v>15</v>
-      </c>
       <c r="C45" s="2" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="E45" s="2" t="s">
-        <v>427</v>
-      </c>
-      <c r="F45" s="2" t="s">
-        <v>428</v>
+        <v>157</v>
+      </c>
+      <c r="E45" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="F45" s="4" t="s">
+        <v>489</v>
       </c>
     </row>
     <row r="46" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B46" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B46" s="2" t="s">
-        <v>15</v>
-      </c>
       <c r="C46" s="2" t="s">
-        <v>368</v>
+        <v>149</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>369</v>
+        <v>150</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>164</v>
+        <v>290</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>165</v>
+        <v>488</v>
       </c>
     </row>
     <row r="47" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B47" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B47" s="2" t="s">
-        <v>15</v>
-      </c>
       <c r="C47" s="2" t="s">
-        <v>155</v>
+        <v>356</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>156</v>
+        <v>357</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>167</v>
+        <v>487</v>
       </c>
     </row>
     <row r="48" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B48" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B48" s="2" t="s">
-        <v>15</v>
-      </c>
       <c r="C48" s="2" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>168</v>
+        <v>376</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>169</v>
+        <v>486</v>
       </c>
     </row>
     <row r="49" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B49" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B49" s="2" t="s">
-        <v>15</v>
-      </c>
       <c r="C49" s="2" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="E49" s="2"/>
-      <c r="F49" s="2"/>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A50" s="3"/>
-      <c r="B50" s="3"/>
-      <c r="C50" s="3"/>
-      <c r="D50" s="3"/>
-      <c r="E50" s="3"/>
-      <c r="F50" s="3"/>
-    </row>
-    <row r="51" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B51" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C51" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="D51" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="E51" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="F51" s="2" t="s">
-        <v>201</v>
-      </c>
+        <v>148</v>
+      </c>
+      <c r="E49" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="F49" s="2" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C50" s="2"/>
+      <c r="D50" s="2"/>
+      <c r="E50" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="F50" s="2" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A51" s="3"/>
+      <c r="B51" s="3"/>
+      <c r="C51" s="3"/>
+      <c r="D51" s="3"/>
+      <c r="E51" s="3"/>
+      <c r="F51" s="3"/>
     </row>
     <row r="52" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B52" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B52" s="2" t="s">
-        <v>17</v>
-      </c>
       <c r="C52" s="2" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="E52" s="4" t="s">
-        <v>202</v>
-      </c>
-      <c r="F52" s="4" t="s">
-        <v>203</v>
+        <v>192</v>
+      </c>
+      <c r="E52" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="F52" s="2" t="s">
+        <v>196</v>
       </c>
     </row>
     <row r="53" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B53" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B53" s="2" t="s">
-        <v>17</v>
-      </c>
       <c r="C53" s="2" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="E53" s="2" t="s">
-        <v>204</v>
-      </c>
-      <c r="F53" s="2" t="s">
-        <v>205</v>
+        <v>182</v>
+      </c>
+      <c r="E53" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="F53" s="4" t="s">
+        <v>198</v>
       </c>
     </row>
     <row r="54" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B54" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B54" s="2" t="s">
-        <v>17</v>
-      </c>
       <c r="C54" s="2" t="s">
-        <v>178</v>
+        <v>360</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>179</v>
+        <v>166</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>183</v>
+        <v>200</v>
       </c>
     </row>
     <row r="55" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B55" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B55" s="2" t="s">
-        <v>17</v>
-      </c>
       <c r="C55" s="2" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>207</v>
+        <v>187</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>208</v>
+        <v>188</v>
       </c>
     </row>
     <row r="56" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B56" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B56" s="2" t="s">
-        <v>17</v>
-      </c>
       <c r="C56" s="2" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
     </row>
     <row r="57" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B57" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B57" s="2" t="s">
-        <v>17</v>
-      </c>
       <c r="C57" s="2" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
     </row>
     <row r="58" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B58" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B58" s="2" t="s">
-        <v>17</v>
-      </c>
       <c r="C58" s="2" t="s">
-        <v>184</v>
+        <v>413</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="E58" s="4" t="s">
-        <v>213</v>
-      </c>
-      <c r="F58" s="4" t="s">
-        <v>214</v>
+        <v>414</v>
+      </c>
+      <c r="E58" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="F58" s="2" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="59" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B59" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B59" s="2" t="s">
-        <v>17</v>
-      </c>
       <c r="C59" s="2" t="s">
-        <v>188</v>
+        <v>179</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="E59" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="F59" s="2" t="s">
-        <v>222</v>
+        <v>180</v>
+      </c>
+      <c r="E59" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="F59" s="4" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="60" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B60" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B60" s="2" t="s">
-        <v>17</v>
-      </c>
       <c r="C60" s="2" t="s">
-        <v>190</v>
+        <v>201</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>191</v>
+        <v>178</v>
       </c>
       <c r="E60" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="F60" s="2" t="s">
         <v>217</v>
-      </c>
-      <c r="F60" s="2" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="61" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B61" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B61" s="2" t="s">
-        <v>17</v>
-      </c>
       <c r="C61" s="2" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>198</v>
+        <v>212</v>
       </c>
       <c r="F61" s="2" t="s">
-        <v>199</v>
+        <v>213</v>
       </c>
     </row>
     <row r="62" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B62" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B62" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C62" s="2" t="s">
+      <c r="C62" s="2"/>
+      <c r="D62" s="2"/>
+      <c r="E62" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="F62" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="D62" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="E62" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="F62" s="2" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A63" s="3"/>
-      <c r="B63" s="3"/>
-      <c r="C63" s="3"/>
-      <c r="D63" s="3"/>
-      <c r="E63" s="3"/>
-      <c r="F63" s="3"/>
+    </row>
+    <row r="63" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A63" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C63" s="2"/>
+      <c r="D63" s="2"/>
+      <c r="E63" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="F63" s="2" t="s">
+        <v>186</v>
+      </c>
     </row>
     <row r="64" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C64" s="2" t="s">
-        <v>223</v>
-      </c>
-      <c r="D64" s="2" t="s">
-        <v>224</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="C64" s="2"/>
+      <c r="D64" s="2"/>
       <c r="E64" s="2" t="s">
-        <v>241</v>
+        <v>162</v>
       </c>
       <c r="F64" s="2" t="s">
-        <v>242</v>
+        <v>163</v>
       </c>
     </row>
     <row r="65" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" s="2" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C65" s="2" t="s">
-        <v>243</v>
-      </c>
-      <c r="D65" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="E65" s="4" t="s">
-        <v>254</v>
-      </c>
-      <c r="F65" s="4" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="66" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A66" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B66" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C66" s="2" t="s">
-        <v>227</v>
-      </c>
-      <c r="D66" s="2" t="s">
-        <v>228</v>
-      </c>
-      <c r="E66" s="2" t="s">
-        <v>244</v>
-      </c>
-      <c r="F66" s="2" t="s">
-        <v>245</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="C65" s="2"/>
+      <c r="D65" s="2"/>
+      <c r="E65" s="2" t="s">
+        <v>354</v>
+      </c>
+      <c r="F65" s="2" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A66" s="3"/>
+      <c r="B66" s="3"/>
+      <c r="C66" s="3"/>
+      <c r="D66" s="3"/>
+      <c r="E66" s="3"/>
+      <c r="F66" s="3"/>
     </row>
     <row r="67" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>229</v>
+        <v>218</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>230</v>
+        <v>219</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
       <c r="F67" s="2" t="s">
-        <v>247</v>
+        <v>237</v>
       </c>
     </row>
     <row r="68" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>231</v>
+        <v>238</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="E68" s="2" t="s">
-        <v>248</v>
-      </c>
-      <c r="F68" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="E68" s="4" t="s">
         <v>249</v>
+      </c>
+      <c r="F68" s="4" t="s">
+        <v>250</v>
       </c>
     </row>
     <row r="69" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A69" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>233</v>
+        <v>100</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>234</v>
+        <v>101</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>250</v>
+        <v>239</v>
       </c>
       <c r="F69" s="2" t="s">
-        <v>251</v>
+        <v>240</v>
       </c>
     </row>
     <row r="70" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>235</v>
+        <v>224</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>236</v>
+        <v>225</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>262</v>
+        <v>241</v>
       </c>
       <c r="F70" s="2" t="s">
-        <v>263</v>
+        <v>242</v>
       </c>
     </row>
     <row r="71" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>237</v>
+        <v>226</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>238</v>
+        <v>227</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>264</v>
+        <v>243</v>
       </c>
       <c r="F71" s="2" t="s">
-        <v>265</v>
+        <v>244</v>
       </c>
     </row>
     <row r="72" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>256</v>
+        <v>245</v>
       </c>
       <c r="F72" s="2" t="s">
-        <v>257</v>
+        <v>246</v>
       </c>
     </row>
     <row r="73" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A73" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C73" s="2"/>
-      <c r="D73" s="2"/>
+        <v>17</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="D73" s="2" t="s">
+        <v>231</v>
+      </c>
       <c r="E73" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="F73" s="2" t="s">
         <v>258</v>
-      </c>
-      <c r="F73" s="2" t="s">
-        <v>259</v>
       </c>
     </row>
     <row r="74" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C74" s="2"/>
-      <c r="D74" s="2"/>
+        <v>17</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="D74" s="2" t="s">
+        <v>233</v>
+      </c>
       <c r="E74" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="F74" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="F74" s="2" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A75" s="3"/>
-      <c r="B75" s="3"/>
-      <c r="C75" s="3"/>
-      <c r="D75" s="3"/>
-      <c r="E75" s="3"/>
-      <c r="F75" s="3"/>
+    </row>
+    <row r="75" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A75" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D75" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="E75" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="F75" s="2" t="s">
+        <v>252</v>
+      </c>
     </row>
     <row r="76" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A76" s="2" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C76" s="2" t="s">
-        <v>270</v>
-      </c>
-      <c r="D76" s="2" t="s">
-        <v>271</v>
-      </c>
-      <c r="E76" s="4" t="s">
-        <v>278</v>
-      </c>
-      <c r="F76" s="4" t="s">
-        <v>279</v>
+        <v>17</v>
+      </c>
+      <c r="C76" s="2"/>
+      <c r="D76" s="2"/>
+      <c r="E76" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="F76" s="2" t="s">
+        <v>254</v>
       </c>
     </row>
     <row r="77" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A77" s="2" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C77" s="2" t="s">
-        <v>268</v>
-      </c>
-      <c r="D77" s="2" t="s">
-        <v>269</v>
-      </c>
+        <v>17</v>
+      </c>
+      <c r="C77" s="2"/>
+      <c r="D77" s="2"/>
       <c r="E77" s="2" t="s">
-        <v>239</v>
+        <v>255</v>
       </c>
       <c r="F77" s="2" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="78" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A78" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B78" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C78" s="2" t="s">
-        <v>266</v>
-      </c>
-      <c r="D78" s="2" t="s">
-        <v>267</v>
-      </c>
-      <c r="E78" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="F78" s="2" t="s">
-        <v>64</v>
-      </c>
+        <v>256</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A78" s="3"/>
+      <c r="B78" s="3"/>
+      <c r="C78" s="3"/>
+      <c r="D78" s="3"/>
+      <c r="E78" s="3"/>
+      <c r="F78" s="3"/>
     </row>
     <row r="79" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A79" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>276</v>
+        <v>265</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>277</v>
-      </c>
-      <c r="E79" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="F79" s="2" t="s">
-        <v>96</v>
+        <v>266</v>
+      </c>
+      <c r="E79" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="F79" s="4" t="s">
+        <v>273</v>
       </c>
     </row>
     <row r="80" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A80" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>274</v>
+        <v>263</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>275</v>
-      </c>
-      <c r="E80" s="2"/>
-      <c r="F80" s="2"/>
-    </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A81" s="3"/>
-      <c r="B81" s="3"/>
-      <c r="C81" s="3"/>
-      <c r="D81" s="3"/>
-      <c r="E81" s="3"/>
-      <c r="F81" s="3"/>
+        <v>264</v>
+      </c>
+      <c r="E80" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="F80" s="2" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A81" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B81" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C81" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="D81" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="E81" s="2" t="s">
+        <v>433</v>
+      </c>
+      <c r="F81" s="2" t="s">
+        <v>434</v>
+      </c>
     </row>
     <row r="82" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A82" s="2" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C82" s="2" t="s">
-        <v>440</v>
-      </c>
-      <c r="D82" s="2" t="s">
-        <v>441</v>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="C82" s="2"/>
+      <c r="D82" s="2"/>
       <c r="E82" s="2" t="s">
-        <v>457</v>
+        <v>94</v>
       </c>
       <c r="F82" s="2" t="s">
-        <v>458</v>
+        <v>95</v>
       </c>
     </row>
     <row r="83" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A83" s="2" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C83" s="2" t="s">
-        <v>462</v>
-      </c>
-      <c r="D83" s="2" t="s">
-        <v>463</v>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="C83" s="2"/>
+      <c r="D83" s="2"/>
       <c r="E83" s="2" t="s">
-        <v>459</v>
+        <v>296</v>
       </c>
       <c r="F83" s="2" t="s">
-        <v>34</v>
+        <v>297</v>
       </c>
     </row>
     <row r="84" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A84" s="2" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C84" s="2" t="s">
-        <v>444</v>
-      </c>
-      <c r="D84" s="2" t="s">
-        <v>445</v>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="C84" s="2"/>
+      <c r="D84" s="2"/>
       <c r="E84" s="2" t="s">
-        <v>460</v>
+        <v>270</v>
       </c>
       <c r="F84" s="2" t="s">
-        <v>461</v>
-      </c>
-    </row>
-    <row r="85" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A85" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B85" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C85" s="2" t="s">
-        <v>446</v>
-      </c>
-      <c r="D85" s="2" t="s">
-        <v>297</v>
-      </c>
-      <c r="E85" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="F85" s="2" t="s">
-        <v>122</v>
-      </c>
+        <v>271</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A85" s="3"/>
+      <c r="B85" s="3"/>
+      <c r="C85" s="3"/>
+      <c r="D85" s="3"/>
+      <c r="E85" s="3"/>
+      <c r="F85" s="3"/>
     </row>
     <row r="86" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A86" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>447</v>
+        <v>426</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>448</v>
+        <v>427</v>
       </c>
       <c r="E86" s="2" t="s">
-        <v>464</v>
+        <v>443</v>
       </c>
       <c r="F86" s="2" t="s">
-        <v>96</v>
+        <v>444</v>
       </c>
     </row>
     <row r="87" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A87" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C87" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="D87" s="2" t="s">
         <v>449</v>
       </c>
-      <c r="D87" s="2" t="s">
-        <v>450</v>
-      </c>
       <c r="E87" s="2" t="s">
-        <v>488</v>
+        <v>464</v>
       </c>
       <c r="F87" s="2" t="s">
-        <v>489</v>
+        <v>465</v>
       </c>
     </row>
     <row r="88" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A88" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>451</v>
+        <v>430</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>452</v>
+        <v>431</v>
       </c>
       <c r="E88" s="2" t="s">
-        <v>480</v>
+        <v>446</v>
       </c>
       <c r="F88" s="2" t="s">
-        <v>481</v>
+        <v>447</v>
       </c>
     </row>
     <row r="89" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A89" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>453</v>
+        <v>432</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>454</v>
+        <v>291</v>
       </c>
       <c r="E89" s="2" t="s">
-        <v>484</v>
+        <v>116</v>
       </c>
       <c r="F89" s="2" t="s">
-        <v>485</v>
+        <v>117</v>
       </c>
     </row>
     <row r="90" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A90" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>455</v>
+        <v>468</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>456</v>
+        <v>469</v>
       </c>
       <c r="E90" s="2" t="s">
-        <v>486</v>
+        <v>450</v>
       </c>
       <c r="F90" s="2" t="s">
-        <v>487</v>
+        <v>95</v>
       </c>
     </row>
     <row r="91" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A91" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>467</v>
+        <v>435</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>58</v>
+        <v>436</v>
       </c>
       <c r="E91" s="2" t="s">
-        <v>490</v>
+        <v>388</v>
       </c>
       <c r="F91" s="2" t="s">
-        <v>491</v>
+        <v>389</v>
       </c>
     </row>
     <row r="92" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A92" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>468</v>
+        <v>437</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>469</v>
+        <v>438</v>
       </c>
       <c r="E92" s="2" t="s">
-        <v>474</v>
+        <v>466</v>
       </c>
       <c r="F92" s="2" t="s">
-        <v>475</v>
+        <v>467</v>
       </c>
     </row>
     <row r="93" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A93" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>470</v>
+        <v>439</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>471</v>
+        <v>440</v>
       </c>
       <c r="E93" s="2" t="s">
-        <v>476</v>
+        <v>462</v>
       </c>
       <c r="F93" s="2" t="s">
-        <v>477</v>
+        <v>463</v>
       </c>
     </row>
     <row r="94" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A94" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>482</v>
+        <v>441</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>483</v>
+        <v>442</v>
       </c>
       <c r="E94" s="2" t="s">
-        <v>478</v>
+        <v>460</v>
       </c>
       <c r="F94" s="2" t="s">
-        <v>479</v>
-      </c>
-    </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A95" s="3"/>
-      <c r="B95" s="3"/>
-      <c r="C95" s="3"/>
-      <c r="D95" s="3"/>
-      <c r="E95" s="3"/>
-      <c r="F95" s="3"/>
+        <v>461</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A95" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B95" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C95" s="2" t="s">
+        <v>456</v>
+      </c>
+      <c r="D95" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="E95" s="2" t="s">
+        <v>476</v>
+      </c>
+      <c r="F95" s="2" t="s">
+        <v>477</v>
+      </c>
     </row>
     <row r="96" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A96" s="2" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C96" s="2" t="s">
-        <v>323</v>
+        <v>454</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>317</v>
-      </c>
-      <c r="E96" s="4" t="s">
-        <v>328</v>
-      </c>
-      <c r="F96" s="4" t="s">
-        <v>329</v>
+        <v>455</v>
+      </c>
+      <c r="E96" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="F96" s="2" t="s">
+        <v>343</v>
       </c>
     </row>
     <row r="97" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A97" s="2" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>314</v>
+        <v>363</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>315</v>
-      </c>
-      <c r="E97" s="2" t="s">
-        <v>330</v>
-      </c>
-      <c r="F97" s="2" t="s">
-        <v>331</v>
-      </c>
+        <v>364</v>
+      </c>
+      <c r="E97" s="2"/>
+      <c r="F97" s="2"/>
     </row>
     <row r="98" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A98" s="2" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>316</v>
+        <v>220</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>317</v>
-      </c>
-      <c r="E98" s="2" t="s">
-        <v>332</v>
-      </c>
-      <c r="F98" s="2" t="s">
-        <v>333</v>
-      </c>
-    </row>
-    <row r="99" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A99" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B99" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C99" s="2" t="s">
-        <v>294</v>
-      </c>
-      <c r="D99" s="2" t="s">
-        <v>295</v>
-      </c>
-      <c r="E99" s="4" t="s">
-        <v>308</v>
-      </c>
-      <c r="F99" s="4" t="s">
-        <v>309</v>
-      </c>
+        <v>221</v>
+      </c>
+      <c r="E98" s="2"/>
+      <c r="F98" s="2"/>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A99" s="3"/>
+      <c r="B99" s="3"/>
+      <c r="C99" s="3"/>
+      <c r="D99" s="3"/>
+      <c r="E99" s="3"/>
+      <c r="F99" s="3"/>
     </row>
     <row r="100" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A100" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C100" s="2" t="s">
-        <v>320</v>
+        <v>308</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>321</v>
+        <v>309</v>
       </c>
       <c r="E100" s="2" t="s">
-        <v>27</v>
+        <v>324</v>
       </c>
       <c r="F100" s="2" t="s">
-        <v>28</v>
+        <v>325</v>
       </c>
     </row>
     <row r="101" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A101" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>66</v>
+        <v>321</v>
       </c>
       <c r="E101" s="2" t="s">
-        <v>304</v>
+        <v>314</v>
       </c>
       <c r="F101" s="2" t="s">
-        <v>305</v>
+        <v>315</v>
       </c>
     </row>
     <row r="102" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A102" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C102" s="2" t="s">
-        <v>312</v>
+        <v>288</v>
       </c>
       <c r="D102" s="2" t="s">
-        <v>313</v>
-      </c>
-      <c r="E102" s="2"/>
-      <c r="F102" s="2"/>
+        <v>289</v>
+      </c>
+      <c r="E102" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="F102" s="4" t="s">
+        <v>303</v>
+      </c>
     </row>
     <row r="103" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A103" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C103" s="2" t="s">
-        <v>324</v>
+        <v>306</v>
       </c>
       <c r="D103" s="2" t="s">
-        <v>325</v>
-      </c>
-      <c r="E103" s="2"/>
-      <c r="F103" s="2"/>
+        <v>307</v>
+      </c>
+      <c r="E103" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F103" s="2" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="104" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A104" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C104" s="2" t="s">
-        <v>326</v>
+        <v>318</v>
       </c>
       <c r="D104" s="2" t="s">
-        <v>327</v>
-      </c>
-      <c r="E104" s="2"/>
-      <c r="F104" s="2"/>
-    </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A105" s="3"/>
-      <c r="B105" s="3"/>
-      <c r="C105" s="3"/>
-      <c r="D105" s="3"/>
-      <c r="E105" s="3"/>
-      <c r="F105" s="3"/>
-    </row>
-    <row r="106" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A106" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B106" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C106" s="2" t="s">
-        <v>336</v>
-      </c>
-      <c r="D106" s="2" t="s">
-        <v>337</v>
-      </c>
-      <c r="E106" s="2" t="s">
-        <v>345</v>
-      </c>
-      <c r="F106" s="2" t="s">
-        <v>346</v>
-      </c>
+        <v>319</v>
+      </c>
+      <c r="E104" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="F104" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A105" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B105" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C105" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="D105" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="E105" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="F105" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A106" s="3"/>
+      <c r="B106" s="3"/>
+      <c r="C106" s="3"/>
+      <c r="D106" s="3"/>
+      <c r="E106" s="3"/>
+      <c r="F106" s="3"/>
     </row>
     <row r="107" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A107" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C107" s="2" t="s">
-        <v>338</v>
-      </c>
-      <c r="D107" s="2" t="s">
-        <v>126</v>
+        <v>21</v>
+      </c>
+      <c r="C107" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="D107" s="9" t="s">
+        <v>481</v>
       </c>
       <c r="E107" s="2" t="s">
-        <v>347</v>
+        <v>337</v>
       </c>
       <c r="F107" s="2" t="s">
-        <v>348</v>
+        <v>490</v>
       </c>
     </row>
     <row r="108" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A108" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C108" s="2" t="s">
-        <v>360</v>
+        <v>331</v>
       </c>
       <c r="D108" s="2" t="s">
-        <v>361</v>
-      </c>
-      <c r="E108" s="4" t="s">
-        <v>381</v>
-      </c>
-      <c r="F108" s="4" t="s">
-        <v>382</v>
+        <v>124</v>
+      </c>
+      <c r="E108" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="F108" s="2" t="s">
+        <v>491</v>
       </c>
     </row>
     <row r="109" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A109" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C109" s="2" t="s">
-        <v>339</v>
+        <v>348</v>
       </c>
       <c r="D109" s="2" t="s">
-        <v>340</v>
-      </c>
-      <c r="E109" s="2" t="s">
-        <v>351</v>
-      </c>
-      <c r="F109" s="2" t="s">
-        <v>352</v>
+        <v>349</v>
+      </c>
+      <c r="E109" s="4" t="s">
+        <v>369</v>
+      </c>
+      <c r="F109" s="4" t="s">
+        <v>492</v>
       </c>
     </row>
     <row r="110" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A110" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>343</v>
+        <v>335</v>
       </c>
       <c r="D110" s="2" t="s">
-        <v>344</v>
+        <v>336</v>
       </c>
       <c r="E110" s="2" t="s">
-        <v>353</v>
+        <v>341</v>
       </c>
       <c r="F110" s="2" t="s">
-        <v>354</v>
+        <v>493</v>
       </c>
     </row>
     <row r="111" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A111" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C111" s="2" t="s">
-        <v>219</v>
-      </c>
-      <c r="D111" s="2" t="s">
-        <v>220</v>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="C111" s="2"/>
+      <c r="D111" s="2"/>
       <c r="E111" s="2" t="s">
-        <v>355</v>
+        <v>332</v>
       </c>
       <c r="F111" s="2" t="s">
-        <v>356</v>
+        <v>494</v>
       </c>
     </row>
     <row r="112" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A112" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C112" s="2"/>
       <c r="D112" s="2"/>
       <c r="E112" s="2" t="s">
-        <v>272</v>
+        <v>344</v>
       </c>
       <c r="F112" s="2" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A113" s="3"/>
-      <c r="B113" s="3"/>
-      <c r="C113" s="3"/>
-      <c r="D113" s="3"/>
-      <c r="E113" s="3"/>
-      <c r="F113" s="3"/>
+        <v>495</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A113" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B113" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C113" s="2"/>
+      <c r="D113" s="2"/>
+      <c r="E113" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="F113" s="2" t="s">
+        <v>496</v>
+      </c>
     </row>
     <row r="114" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A114" s="2" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C114" s="2" t="s">
-        <v>357</v>
-      </c>
-      <c r="D114" s="2" t="s">
-        <v>218</v>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="C114" s="2"/>
+      <c r="D114" s="2"/>
       <c r="E114" s="2" t="s">
-        <v>375</v>
+        <v>330</v>
       </c>
       <c r="F114" s="2" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="115" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A115" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B115" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C115" s="2" t="s">
-        <v>358</v>
-      </c>
-      <c r="D115" s="2" t="s">
-        <v>359</v>
-      </c>
-      <c r="E115" s="2" t="s">
-        <v>377</v>
-      </c>
-      <c r="F115" s="2" t="s">
-        <v>378</v>
-      </c>
+        <v>497</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A115" s="3"/>
+      <c r="B115" s="3"/>
+      <c r="C115" s="3"/>
+      <c r="D115" s="3"/>
+      <c r="E115" s="3"/>
+      <c r="F115" s="3"/>
     </row>
     <row r="116" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A116" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C116" s="2" t="s">
-        <v>362</v>
+        <v>345</v>
       </c>
       <c r="D116" s="2" t="s">
-        <v>363</v>
+        <v>213</v>
       </c>
       <c r="E116" s="2" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="F116" s="2" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
     </row>
     <row r="117" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A117" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B117" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C117" s="2" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
       <c r="D117" s="2" t="s">
-        <v>342</v>
-      </c>
-      <c r="E117" s="4" t="s">
-        <v>349</v>
-      </c>
-      <c r="F117" s="4" t="s">
-        <v>350</v>
+        <v>347</v>
+      </c>
+      <c r="E117" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="F117" s="2" t="s">
+        <v>366</v>
       </c>
     </row>
     <row r="118" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A118" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C118" s="2" t="s">
-        <v>364</v>
+        <v>350</v>
       </c>
       <c r="D118" s="2" t="s">
-        <v>365</v>
+        <v>351</v>
       </c>
       <c r="E118" s="2" t="s">
-        <v>383</v>
+        <v>367</v>
       </c>
       <c r="F118" s="2" t="s">
-        <v>384</v>
+        <v>368</v>
       </c>
     </row>
     <row r="119" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A119" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B119" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C119" s="2" t="s">
-        <v>366</v>
+        <v>333</v>
       </c>
       <c r="D119" s="2" t="s">
-        <v>367</v>
-      </c>
-      <c r="E119" s="2" t="s">
-        <v>385</v>
-      </c>
-      <c r="F119" s="2" t="s">
-        <v>386</v>
+        <v>334</v>
+      </c>
+      <c r="E119" s="4" t="s">
+        <v>339</v>
+      </c>
+      <c r="F119" s="4" t="s">
+        <v>340</v>
       </c>
     </row>
     <row r="120" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A120" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C120" s="2" t="s">
-        <v>373</v>
+        <v>352</v>
       </c>
       <c r="D120" s="2" t="s">
-        <v>374</v>
+        <v>353</v>
       </c>
       <c r="E120" s="2" t="s">
-        <v>387</v>
+        <v>370</v>
       </c>
       <c r="F120" s="2" t="s">
-        <v>388</v>
+        <v>371</v>
       </c>
     </row>
     <row r="121" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A121" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C121" s="2" t="s">
-        <v>370</v>
+        <v>247</v>
       </c>
       <c r="D121" s="2" t="s">
-        <v>371</v>
+        <v>248</v>
       </c>
       <c r="E121" s="2" t="s">
-        <v>389</v>
+        <v>372</v>
       </c>
       <c r="F121" s="2" t="s">
-        <v>390</v>
+        <v>373</v>
       </c>
     </row>
     <row r="122" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A122" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>372</v>
+        <v>361</v>
       </c>
       <c r="D122" s="2" t="s">
-        <v>171</v>
+        <v>362</v>
       </c>
       <c r="E122" s="2" t="s">
-        <v>391</v>
+        <v>379</v>
       </c>
       <c r="F122" s="2" t="s">
-        <v>392</v>
+        <v>371</v>
       </c>
     </row>
     <row r="123" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A123" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C123" s="2" t="s">
-        <v>252</v>
+        <v>358</v>
       </c>
       <c r="D123" s="2" t="s">
-        <v>253</v>
+        <v>359</v>
       </c>
       <c r="E123" s="2" t="s">
-        <v>393</v>
+        <v>268</v>
       </c>
       <c r="F123" s="2" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A124" s="3"/>
-      <c r="B124" s="3"/>
-      <c r="C124" s="3"/>
-      <c r="D124" s="3"/>
-      <c r="E124" s="3"/>
-      <c r="F124" s="3"/>
+        <v>269</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A124" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B124" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C124" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="D124" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="E124" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="F124" s="2" t="s">
+        <v>375</v>
+      </c>
     </row>
     <row r="125" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A125" s="2" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C125" s="2" t="s">
-        <v>394</v>
-      </c>
-      <c r="D125" s="2" t="s">
-        <v>395</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="C125" s="2"/>
+      <c r="D125" s="2"/>
       <c r="E125" s="2" t="s">
-        <v>417</v>
+        <v>472</v>
       </c>
       <c r="F125" s="2" t="s">
-        <v>418</v>
-      </c>
-    </row>
-    <row r="126" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A126" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B126" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C126" s="2" t="s">
-        <v>415</v>
-      </c>
-      <c r="D126" s="2" t="s">
-        <v>416</v>
-      </c>
-      <c r="E126" s="2" t="s">
-        <v>432</v>
-      </c>
-      <c r="F126" s="2" t="s">
-        <v>433</v>
-      </c>
+        <v>473</v>
+      </c>
+    </row>
+    <row r="126" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A126" s="3"/>
+      <c r="B126" s="3"/>
+      <c r="C126" s="3"/>
+      <c r="D126" s="3"/>
+      <c r="E126" s="3"/>
+      <c r="F126" s="3"/>
     </row>
     <row r="127" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A127" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C127" s="2" t="s">
-        <v>398</v>
+        <v>380</v>
       </c>
       <c r="D127" s="2" t="s">
-        <v>399</v>
+        <v>381</v>
       </c>
       <c r="E127" s="2" t="s">
-        <v>421</v>
+        <v>86</v>
       </c>
       <c r="F127" s="2" t="s">
-        <v>422</v>
+        <v>87</v>
       </c>
     </row>
     <row r="128" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A128" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C128" s="2" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="D128" s="2" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="E128" s="2" t="s">
-        <v>423</v>
+        <v>416</v>
       </c>
       <c r="F128" s="2" t="s">
-        <v>424</v>
+        <v>417</v>
       </c>
     </row>
     <row r="129" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A129" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C129" s="2" t="s">
-        <v>402</v>
+        <v>384</v>
       </c>
       <c r="D129" s="2" t="s">
-        <v>403</v>
+        <v>385</v>
       </c>
       <c r="E129" s="2" t="s">
-        <v>425</v>
+        <v>407</v>
       </c>
       <c r="F129" s="2" t="s">
-        <v>426</v>
+        <v>408</v>
       </c>
     </row>
     <row r="130" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A130" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C130" s="2" t="s">
-        <v>404</v>
+        <v>386</v>
       </c>
       <c r="D130" s="2" t="s">
-        <v>405</v>
+        <v>387</v>
       </c>
       <c r="E130" s="2" t="s">
-        <v>434</v>
+        <v>409</v>
       </c>
       <c r="F130" s="2" t="s">
-        <v>435</v>
+        <v>410</v>
       </c>
     </row>
     <row r="131" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A131" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C131" s="2" t="s">
-        <v>406</v>
+        <v>298</v>
       </c>
       <c r="D131" s="2" t="s">
-        <v>199</v>
+        <v>299</v>
       </c>
       <c r="E131" s="2" t="s">
-        <v>429</v>
+        <v>411</v>
       </c>
       <c r="F131" s="2" t="s">
-        <v>66</v>
+        <v>412</v>
       </c>
     </row>
     <row r="132" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A132" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C132" s="2" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="D132" s="2" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="E132" s="2" t="s">
-        <v>430</v>
+        <v>62</v>
       </c>
       <c r="F132" s="2" t="s">
-        <v>431</v>
+        <v>63</v>
       </c>
     </row>
     <row r="133" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A133" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B133" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C133" s="2" t="s">
-        <v>413</v>
+        <v>392</v>
       </c>
       <c r="D133" s="2" t="s">
-        <v>414</v>
-      </c>
-      <c r="E133" s="2"/>
-      <c r="F133" s="2"/>
+        <v>194</v>
+      </c>
+      <c r="E133" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F133" s="2" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="134" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A134" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B134" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C134" s="2" t="s">
-        <v>411</v>
+        <v>393</v>
       </c>
       <c r="D134" s="2" t="s">
-        <v>412</v>
-      </c>
-      <c r="E134" s="2"/>
-      <c r="F134" s="2"/>
+        <v>394</v>
+      </c>
+      <c r="E134" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="F134" s="2" t="s">
+        <v>391</v>
+      </c>
     </row>
     <row r="135" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A135" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B135" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C135" s="2" t="s">
-        <v>419</v>
+        <v>399</v>
       </c>
       <c r="D135" s="2" t="s">
-        <v>420</v>
+        <v>400</v>
       </c>
       <c r="E135" s="2"/>
       <c r="F135" s="2"/>
     </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A136" s="3"/>
-      <c r="B136" s="3"/>
-      <c r="C136" s="3"/>
-      <c r="D136" s="3"/>
-      <c r="E136" s="3"/>
-      <c r="F136" s="3"/>
-    </row>
-    <row r="137" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A137" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B137" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C137" s="2" t="s">
-        <v>280</v>
-      </c>
-      <c r="D137" s="2" t="s">
-        <v>281</v>
-      </c>
-      <c r="E137" s="2" t="s">
-        <v>296</v>
-      </c>
-      <c r="F137" s="2" t="s">
-        <v>297</v>
-      </c>
+    <row r="136" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A136" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B136" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C136" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="D136" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="E136" s="2"/>
+      <c r="F136" s="2"/>
+    </row>
+    <row r="137" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A137" s="3"/>
+      <c r="B137" s="3"/>
+      <c r="C137" s="3"/>
+      <c r="D137" s="3"/>
+      <c r="E137" s="3"/>
+      <c r="F137" s="3"/>
     </row>
     <row r="138" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A138" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B138" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C138" s="2" t="s">
-        <v>282</v>
+        <v>317</v>
       </c>
       <c r="D138" s="2" t="s">
-        <v>283</v>
-      </c>
-      <c r="E138" s="2" t="s">
-        <v>298</v>
-      </c>
-      <c r="F138" s="2" t="s">
-        <v>299</v>
+        <v>311</v>
+      </c>
+      <c r="E138" s="4" t="s">
+        <v>322</v>
+      </c>
+      <c r="F138" s="4" t="s">
+        <v>323</v>
       </c>
     </row>
     <row r="139" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A139" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C139" s="2" t="s">
-        <v>284</v>
+        <v>310</v>
       </c>
       <c r="D139" s="2" t="s">
-        <v>285</v>
+        <v>311</v>
       </c>
       <c r="E139" s="2" t="s">
-        <v>300</v>
+        <v>280</v>
       </c>
       <c r="F139" s="2" t="s">
-        <v>301</v>
+        <v>281</v>
       </c>
     </row>
     <row r="140" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A140" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C140" s="2" t="s">
-        <v>286</v>
+        <v>276</v>
       </c>
       <c r="D140" s="2" t="s">
-        <v>287</v>
+        <v>277</v>
       </c>
       <c r="E140" s="2" t="s">
-        <v>302</v>
+        <v>292</v>
       </c>
       <c r="F140" s="2" t="s">
-        <v>303</v>
+        <v>293</v>
       </c>
     </row>
     <row r="141" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A141" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B141" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C141" s="2" t="s">
-        <v>318</v>
+        <v>278</v>
       </c>
       <c r="D141" s="2" t="s">
-        <v>319</v>
-      </c>
-      <c r="E141" s="4" t="s">
-        <v>334</v>
-      </c>
-      <c r="F141" s="4" t="s">
-        <v>335</v>
+        <v>279</v>
+      </c>
+      <c r="E141" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="F141" s="2" t="s">
+        <v>295</v>
       </c>
     </row>
     <row r="142" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A142" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B142" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C142" s="2" t="s">
-        <v>290</v>
+        <v>382</v>
       </c>
       <c r="D142" s="2" t="s">
-        <v>291</v>
+        <v>383</v>
       </c>
       <c r="E142" s="2" t="s">
-        <v>306</v>
+        <v>300</v>
       </c>
       <c r="F142" s="2" t="s">
-        <v>307</v>
+        <v>301</v>
       </c>
     </row>
     <row r="143" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A143" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B143" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C143" s="2" t="s">
-        <v>292</v>
+        <v>312</v>
       </c>
       <c r="D143" s="2" t="s">
-        <v>293</v>
-      </c>
-      <c r="E143" s="2" t="s">
-        <v>310</v>
-      </c>
-      <c r="F143" s="2" t="s">
-        <v>311</v>
+        <v>313</v>
+      </c>
+      <c r="E143" s="4" t="s">
+        <v>328</v>
+      </c>
+      <c r="F143" s="4" t="s">
+        <v>329</v>
       </c>
     </row>
     <row r="144" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A144" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C144" s="2" t="s">
-        <v>396</v>
+        <v>282</v>
       </c>
       <c r="D144" s="2" t="s">
-        <v>397</v>
+        <v>283</v>
       </c>
       <c r="E144" s="2"/>
       <c r="F144" s="2"/>
     </row>
     <row r="145" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A145" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B145" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C145" s="2" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="D145" s="2" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="E145" s="2"/>
       <c r="F145" s="2"/>
     </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A146" s="3"/>
-      <c r="B146" s="3"/>
-      <c r="C146" s="3"/>
-      <c r="D146" s="3"/>
-      <c r="E146" s="3"/>
-      <c r="F146" s="3"/>
-    </row>
-    <row r="147" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A147" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B147" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C147" s="2" t="s">
-        <v>472</v>
-      </c>
-      <c r="D147" s="2" t="s">
-        <v>473</v>
-      </c>
-      <c r="E147" s="2" t="s">
-        <v>465</v>
-      </c>
-      <c r="F147" s="2" t="s">
-        <v>466</v>
-      </c>
+    <row r="146" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A146" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B146" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C146" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="D146" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="E146" s="2"/>
+      <c r="F146" s="2"/>
+    </row>
+    <row r="147" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A147" s="3"/>
+      <c r="B147" s="3"/>
+      <c r="C147" s="3"/>
+      <c r="D147" s="3"/>
+      <c r="E147" s="3"/>
+      <c r="F147" s="3"/>
     </row>
     <row r="148" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A148" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C148" s="2" t="s">
-        <v>436</v>
+        <v>458</v>
       </c>
       <c r="D148" s="2" t="s">
-        <v>437</v>
+        <v>459</v>
       </c>
       <c r="E148" s="2" t="s">
-        <v>492</v>
+        <v>451</v>
       </c>
       <c r="F148" s="2" t="s">
-        <v>493</v>
+        <v>452</v>
       </c>
     </row>
     <row r="149" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A149" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B149" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C149" s="2" t="s">
-        <v>438</v>
+        <v>422</v>
       </c>
       <c r="D149" s="2" t="s">
-        <v>439</v>
-      </c>
-      <c r="E149" s="2"/>
-      <c r="F149" s="2"/>
-    </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A150" s="3"/>
-      <c r="B150" s="3"/>
-      <c r="C150" s="3"/>
-      <c r="D150" s="3"/>
-      <c r="E150" s="3"/>
-      <c r="F150" s="3"/>
+        <v>423</v>
+      </c>
+      <c r="E149" s="2" t="s">
+        <v>478</v>
+      </c>
+      <c r="F149" s="2" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="150" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A150" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B150" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C150" s="2" t="s">
+        <v>453</v>
+      </c>
+      <c r="D150" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="E150" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="F150" s="2" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="151" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A151" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B151" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C151" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="D151" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="E151" s="2" t="s">
+        <v>470</v>
+      </c>
+      <c r="F151" s="2" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="152" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A152" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B152" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C152" s="2" t="s">
+        <v>474</v>
+      </c>
+      <c r="D152" s="2" t="s">
+        <v>475</v>
+      </c>
+      <c r="E152" s="2"/>
+      <c r="F152" s="2"/>
+    </row>
+    <row r="153" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A153" s="3"/>
+      <c r="B153" s="3"/>
+      <c r="C153" s="3"/>
+      <c r="D153" s="3"/>
+      <c r="E153" s="3"/>
+      <c r="F153" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Fall 2025 Mid 2
</commit_message>
<xml_diff>
--- a/backend/data/mid1.xlsx
+++ b/backend/data/mid1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{61C495D2-2E65-4DA4-B664-46CA9A734B33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4CE3A689-DB91-4AE4-8BB0-1F7F28A50B1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B8B9A0B7-7B4A-4757-82D6-2903DF6C0B7B}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C58E2495-2073-4214-BC36-B2DEB58F93ED}"/>
   </bookViews>
   <sheets>
     <sheet name="Complete" sheetId="5" r:id="rId1"/>
@@ -20,7 +20,9 @@
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
         <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
@@ -31,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="322">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="369">
   <si>
     <t>Fall 2025 Semester</t>
   </si>
@@ -66,27 +68,15 @@
     <t>Saturday</t>
   </si>
   <si>
-    <t>20-Sep-2025</t>
-  </si>
-  <si>
     <t>Monday</t>
   </si>
   <si>
-    <t>22-Sep-2025</t>
-  </si>
-  <si>
     <t>Tuesday</t>
   </si>
   <si>
-    <t>23-Sep-2025</t>
-  </si>
-  <si>
     <t>Wednesday</t>
   </si>
   <si>
-    <t>24-Sep-2025</t>
-  </si>
-  <si>
     <t>ME2002</t>
   </si>
   <si>
@@ -237,9 +227,6 @@
     <t>Decision Science for Business</t>
   </si>
   <si>
-    <t>ME1001</t>
-  </si>
-  <si>
     <t>Engineering Drawing</t>
   </si>
   <si>
@@ -996,14 +983,170 @@
     <t>Contracts</t>
   </si>
   <si>
-    <t>COMPLETE DATE SHEET - MIDTERM - I               StuV1.2</t>
+    <t>MG5050</t>
+  </si>
+  <si>
+    <t>Econometrics</t>
+  </si>
+  <si>
+    <t>CS5059</t>
+  </si>
+  <si>
+    <t>Database System</t>
+  </si>
+  <si>
+    <t>AF4001</t>
+  </si>
+  <si>
+    <t>Accounting for Managers</t>
+  </si>
+  <si>
+    <t>BA5003</t>
+  </si>
+  <si>
+    <t>Predictive Modelling</t>
+  </si>
+  <si>
+    <t>AF5001</t>
+  </si>
+  <si>
+    <t>Applied Corporate Finance</t>
+  </si>
+  <si>
+    <t>AF5003</t>
+  </si>
+  <si>
+    <t>Financial Reporting and Analysis</t>
+  </si>
+  <si>
+    <t>BA5002</t>
+  </si>
+  <si>
+    <t>Data Driven Decision Making and Optimization</t>
+  </si>
+  <si>
+    <t>BA5005</t>
+  </si>
+  <si>
+    <t>Applied Calculus for Business</t>
+  </si>
+  <si>
+    <t>MG4004</t>
+  </si>
+  <si>
+    <t>Applied Statistics for Business</t>
+  </si>
+  <si>
+    <t>MG4002</t>
+  </si>
+  <si>
+    <t>Communication for Managers</t>
+  </si>
+  <si>
+    <t>MG4010</t>
+  </si>
+  <si>
+    <t>Marketing</t>
+  </si>
+  <si>
+    <t>MG5015</t>
+  </si>
+  <si>
+    <t>Strategic HR and Leadership</t>
+  </si>
+  <si>
+    <t>MG5006</t>
+  </si>
+  <si>
+    <t>Marketing Analytics</t>
+  </si>
+  <si>
+    <t>MG4006</t>
+  </si>
+  <si>
+    <t>Management and Org. Behaviour</t>
+  </si>
+  <si>
+    <t>BA5006</t>
+  </si>
+  <si>
+    <t>Advanced Data Analysis</t>
+  </si>
+  <si>
+    <t>MG4005</t>
+  </si>
+  <si>
+    <t>Business Economics for Managers</t>
+  </si>
+  <si>
+    <t>MG5011</t>
+  </si>
+  <si>
+    <t>Advanced Research Methods</t>
+  </si>
+  <si>
+    <t>MG5034</t>
+  </si>
+  <si>
+    <t>Recruitment and Selection</t>
+  </si>
+  <si>
+    <t>MG5031</t>
+  </si>
+  <si>
+    <t>Business Processes using SAP</t>
+  </si>
+  <si>
+    <t>AF4010</t>
+  </si>
+  <si>
+    <t>Accounting and Finance for Managers</t>
+  </si>
+  <si>
+    <t>CS4089</t>
+  </si>
+  <si>
+    <t>Programming for Business Applications</t>
+  </si>
+  <si>
+    <t>MG5055</t>
+  </si>
+  <si>
+    <t>Ethics in Business Analytics</t>
+  </si>
+  <si>
+    <t>MG5017</t>
+  </si>
+  <si>
+    <t>Strategic Marketing</t>
+  </si>
+  <si>
+    <t>MG5024</t>
+  </si>
+  <si>
+    <t>Cases in Management</t>
+  </si>
+  <si>
+    <t>01-Nov-2025</t>
+  </si>
+  <si>
+    <t>03-Nov-2025</t>
+  </si>
+  <si>
+    <t>04-Nov-2025</t>
+  </si>
+  <si>
+    <t>05-Nov-2025</t>
+  </si>
+  <si>
+    <t>COMPLETE DATE SHEET - II</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -1017,28 +1160,32 @@
       <sz val="18"/>
       <color indexed="10"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color indexed="8"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
       <b/>
       <i/>
       <sz val="14"/>
-      <color indexed="23"/>
+      <color theme="1"/>
       <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color indexed="8"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color indexed="8"/>
-      <name val="Calibri"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -1062,7 +1209,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
+        <fgColor theme="5" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1103,23 +1250,26 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1455,64 +1605,64 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20F9AE8E-B2C8-4772-8A83-92B4FCD1E788}">
-  <dimension ref="A1:O42"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E539384B-9327-404B-83FE-E84881B34C8F}">
+  <dimension ref="A1:O51"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="7.88671875" customWidth="1"/>
-    <col min="4" max="4" width="16.44140625" customWidth="1"/>
+    <col min="4" max="4" width="17" customWidth="1"/>
     <col min="5" max="5" width="7.6640625" customWidth="1"/>
-    <col min="6" max="6" width="16.44140625" customWidth="1"/>
+    <col min="6" max="6" width="14.33203125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="7.6640625" customWidth="1"/>
-    <col min="8" max="8" width="16.44140625" customWidth="1"/>
+    <col min="8" max="8" width="14.33203125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="8.109375" customWidth="1"/>
-    <col min="10" max="10" width="16.44140625" customWidth="1"/>
+    <col min="10" max="10" width="14.33203125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="8.109375" customWidth="1"/>
-    <col min="12" max="12" width="16.44140625" customWidth="1"/>
+    <col min="12" max="12" width="14.33203125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="7.88671875" customWidth="1"/>
-    <col min="14" max="14" width="16.44140625" customWidth="1"/>
+    <col min="14" max="14" width="14.33203125" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="22.8" x14ac:dyDescent="0.4">
-      <c r="A1" s="6" t="s">
-        <v>321</v>
-      </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
-      <c r="J1" s="6"/>
-      <c r="K1" s="6"/>
-      <c r="L1" s="6"/>
-      <c r="M1" s="6"/>
-      <c r="N1" s="6"/>
-      <c r="O1" s="5"/>
+      <c r="A1" s="7" t="s">
+        <v>368</v>
+      </c>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="7"/>
+      <c r="J1" s="7"/>
+      <c r="K1" s="7"/>
+      <c r="L1" s="7"/>
+      <c r="M1" s="7"/>
+      <c r="N1" s="7"/>
+      <c r="O1" s="6"/>
     </row>
     <row r="2" spans="1:15" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="7"/>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="7"/>
-      <c r="J2" s="7"/>
-      <c r="K2" s="7"/>
-      <c r="L2" s="7"/>
-      <c r="M2" s="7"/>
-      <c r="N2" s="7"/>
-      <c r="O2" s="5"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8"/>
+      <c r="I2" s="8"/>
+      <c r="J2" s="8"/>
+      <c r="K2" s="8"/>
+      <c r="L2" s="8"/>
+      <c r="M2" s="8"/>
+      <c r="N2" s="8"/>
+      <c r="O2" s="6"/>
     </row>
     <row r="3" spans="1:15" ht="32.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
@@ -1562,1393 +1712,1665 @@
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>11</v>
+      <c r="B4" s="5" t="s">
+        <v>364</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5" spans="1:15" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>11</v>
+      <c r="B5" s="5" t="s">
+        <v>364</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="L5" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="M5" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="M5" s="2" t="s">
-        <v>80</v>
-      </c>
       <c r="N5" s="2" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
     </row>
     <row r="6" spans="1:15" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>11</v>
+      <c r="B6" s="5" t="s">
+        <v>364</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="I6" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="M6" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="N6" s="2" t="s">
         <v>78</v>
-      </c>
-      <c r="J6" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="K6" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="L6" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="M6" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="N6" s="2" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="7" spans="1:15" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>11</v>
+      <c r="B7" s="5" t="s">
+        <v>364</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="8" spans="1:15" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>11</v>
+      <c r="B8" s="5" t="s">
+        <v>364</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="K8" s="2"/>
-      <c r="L8" s="2"/>
+        <v>47</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>319</v>
+      </c>
       <c r="M8" s="2" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9" spans="1:15" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>11</v>
+      <c r="B9" s="5" t="s">
+        <v>364</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>302</v>
+        <v>297</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
       <c r="I9" s="2" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="K9" s="2"/>
       <c r="L9" s="2"/>
       <c r="M9" s="2" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
     </row>
     <row r="10" spans="1:15" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>11</v>
+      <c r="B10" s="5" t="s">
+        <v>364</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>303</v>
-      </c>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
+        <v>298</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>317</v>
+      </c>
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
       <c r="I10" s="2" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="K10" s="2"/>
       <c r="L10" s="2"/>
-      <c r="M10" s="2"/>
-      <c r="N10" s="2"/>
+      <c r="M10" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="N10" s="2" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="11" spans="1:15" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="2" t="s">
-        <v>11</v>
+      <c r="B11" s="5" t="s">
+        <v>364</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="E11" s="2"/>
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
-      <c r="I11" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="J11" s="2" t="s">
-        <v>85</v>
-      </c>
+      <c r="I11" s="2"/>
+      <c r="J11" s="2"/>
       <c r="K11" s="2"/>
       <c r="L11" s="2"/>
-      <c r="M11" s="2"/>
-      <c r="N11" s="2"/>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A12" s="3"/>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-      <c r="I12" s="3"/>
-      <c r="J12" s="3"/>
-      <c r="K12" s="3"/>
-      <c r="L12" s="3"/>
-      <c r="M12" s="3"/>
-      <c r="N12" s="3"/>
+      <c r="M11" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="N11" s="2" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>364</v>
+      </c>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+      <c r="I12" s="2"/>
+      <c r="J12" s="2"/>
+      <c r="K12" s="2"/>
+      <c r="L12" s="2"/>
+      <c r="M12" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="N12" s="2" t="s">
+        <v>325</v>
+      </c>
     </row>
     <row r="13" spans="1:15" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="I13" s="4" t="s">
-        <v>317</v>
-      </c>
-      <c r="J13" s="4" t="s">
-        <v>318</v>
-      </c>
-      <c r="K13" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="L13" s="2" t="s">
-        <v>138</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>364</v>
+      </c>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
+      <c r="I13" s="2"/>
+      <c r="J13" s="2"/>
+      <c r="K13" s="2"/>
+      <c r="L13" s="2"/>
       <c r="M13" s="2" t="s">
-        <v>146</v>
+        <v>326</v>
       </c>
       <c r="N13" s="2" t="s">
-        <v>147</v>
+        <v>327</v>
       </c>
     </row>
     <row r="14" spans="1:15" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="H14" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="I14" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="J14" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="K14" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="L14" s="2" t="s">
-        <v>141</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>364</v>
+      </c>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
+      <c r="I14" s="2"/>
+      <c r="J14" s="2"/>
+      <c r="K14" s="2"/>
+      <c r="L14" s="2"/>
       <c r="M14" s="2" t="s">
-        <v>148</v>
+        <v>328</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="15" spans="1:15" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="G15" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="H15" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="I15" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="J15" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="K15" s="2" t="s">
-        <v>290</v>
-      </c>
-      <c r="L15" s="2" t="s">
-        <v>291</v>
-      </c>
-      <c r="M15" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="N15" s="2" t="s">
-        <v>151</v>
-      </c>
+        <v>329</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A15" s="3"/>
+      <c r="B15" s="3"/>
+      <c r="C15" s="3"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="3"/>
+      <c r="I15" s="3"/>
+      <c r="J15" s="3"/>
+      <c r="K15" s="3"/>
+      <c r="L15" s="3"/>
+      <c r="M15" s="3"/>
+      <c r="N15" s="3"/>
     </row>
     <row r="16" spans="1:15" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>365</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>104</v>
+        <v>161</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>105</v>
+        <v>162</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="I16" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="J16" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="I16" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="J16" s="4" t="s">
+        <v>313</v>
+      </c>
+      <c r="K16" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="K16" s="2"/>
-      <c r="L16" s="2"/>
+      <c r="L16" s="2" t="s">
+        <v>133</v>
+      </c>
       <c r="M16" s="2" t="s">
-        <v>152</v>
+        <v>141</v>
       </c>
       <c r="N16" s="2" t="s">
-        <v>153</v>
+        <v>142</v>
       </c>
     </row>
     <row r="17" spans="1:14" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>365</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>20</v>
+        <v>91</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>21</v>
+        <v>57</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>174</v>
+        <v>107</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>121</v>
+        <v>112</v>
       </c>
       <c r="H17" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="I17" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="I17" s="2" t="s">
-        <v>133</v>
-      </c>
       <c r="J17" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="K17" s="2"/>
-      <c r="L17" s="2"/>
+        <v>123</v>
+      </c>
+      <c r="K17" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="L17" s="2" t="s">
+        <v>136</v>
+      </c>
       <c r="M17" s="2" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="N17" s="2" t="s">
-        <v>155</v>
+        <v>144</v>
       </c>
     </row>
     <row r="18" spans="1:14" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>365</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>144</v>
+        <v>92</v>
       </c>
       <c r="D18" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="J18" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="K18" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="L18" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="M18" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="E18" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="G18" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="H18" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="I18" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="J18" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="K18" s="2"/>
-      <c r="L18" s="2"/>
-      <c r="M18" s="2" t="s">
-        <v>156</v>
-      </c>
       <c r="N18" s="2" t="s">
-        <v>157</v>
+        <v>146</v>
       </c>
     </row>
     <row r="19" spans="1:14" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>365</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>279</v>
+        <v>94</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>280</v>
+        <v>95</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="G19" s="2"/>
-      <c r="H19" s="2"/>
+        <v>100</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>117</v>
+      </c>
       <c r="I19" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="K19" s="2"/>
-      <c r="L19" s="2"/>
+        <v>127</v>
+      </c>
+      <c r="K19" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="L19" s="2" t="s">
+        <v>331</v>
+      </c>
       <c r="M19" s="2" t="s">
-        <v>158</v>
+        <v>147</v>
       </c>
       <c r="N19" s="2" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="20" spans="1:14" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
+        <v>11</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>365</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>17</v>
+      </c>
       <c r="E20" s="2" t="s">
-        <v>315</v>
+        <v>169</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>316</v>
-      </c>
-      <c r="G20" s="2"/>
-      <c r="H20" s="2"/>
-      <c r="I20" s="2"/>
-      <c r="J20" s="2"/>
-      <c r="K20" s="2"/>
-      <c r="L20" s="2"/>
+        <v>104</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="I20" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="J20" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="K20" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="L20" s="2" t="s">
+        <v>333</v>
+      </c>
       <c r="M20" s="2" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="N20" s="2" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
     </row>
     <row r="21" spans="1:14" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
+        <v>11</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>365</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>104</v>
+      </c>
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
-      <c r="I21" s="2"/>
-      <c r="J21" s="2"/>
-      <c r="K21" s="2"/>
-      <c r="L21" s="2"/>
+      <c r="I21" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="J21" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="K21" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="L21" s="2" t="s">
+        <v>335</v>
+      </c>
       <c r="M21" s="2" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="N21" s="2" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A22" s="3"/>
-      <c r="B22" s="3"/>
-      <c r="C22" s="3"/>
-      <c r="D22" s="3"/>
-      <c r="E22" s="3"/>
-      <c r="F22" s="3"/>
-      <c r="G22" s="3"/>
-      <c r="H22" s="3"/>
-      <c r="I22" s="3"/>
-      <c r="J22" s="3"/>
-      <c r="K22" s="3"/>
-      <c r="L22" s="3"/>
-      <c r="M22" s="3"/>
-      <c r="N22" s="3"/>
+        <v>152</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>365</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="G22" s="2"/>
+      <c r="H22" s="2"/>
+      <c r="I22" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="J22" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="K22" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="L22" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="M22" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="N22" s="2" t="s">
+        <v>154</v>
+      </c>
     </row>
     <row r="23" spans="1:14" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>163</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>365</v>
+      </c>
+      <c r="C23" s="2"/>
+      <c r="D23" s="2"/>
       <c r="E23" s="2" t="s">
-        <v>186</v>
+        <v>310</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="G23" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="H23" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="I23" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="J23" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="K23" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="L23" s="2" t="s">
-        <v>210</v>
-      </c>
+        <v>311</v>
+      </c>
+      <c r="G23" s="2"/>
+      <c r="H23" s="2"/>
+      <c r="I23" s="2"/>
+      <c r="J23" s="2"/>
+      <c r="K23" s="2"/>
+      <c r="L23" s="2"/>
       <c r="M23" s="2" t="s">
-        <v>219</v>
+        <v>155</v>
       </c>
       <c r="N23" s="2" t="s">
-        <v>220</v>
+        <v>156</v>
       </c>
     </row>
     <row r="24" spans="1:14" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>165</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>365</v>
+      </c>
+      <c r="C24" s="2"/>
+      <c r="D24" s="2"/>
       <c r="E24" s="2" t="s">
-        <v>76</v>
+        <v>263</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="G24" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="H24" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="I24" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="J24" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="K24" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="L24" s="2" t="s">
-        <v>212</v>
-      </c>
+        <v>264</v>
+      </c>
+      <c r="G24" s="2"/>
+      <c r="H24" s="2"/>
+      <c r="I24" s="2"/>
+      <c r="J24" s="2"/>
+      <c r="K24" s="2"/>
+      <c r="L24" s="2"/>
       <c r="M24" s="2" t="s">
-        <v>221</v>
+        <v>137</v>
       </c>
       <c r="N24" s="2" t="s">
-        <v>222</v>
+        <v>138</v>
       </c>
     </row>
     <row r="25" spans="1:14" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="G25" s="2" t="s">
-        <v>193</v>
-      </c>
-      <c r="H25" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="I25" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="J25" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="K25" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="L25" s="2" t="s">
-        <v>23</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>365</v>
+      </c>
+      <c r="C25" s="2"/>
+      <c r="D25" s="2"/>
+      <c r="E25" s="2"/>
+      <c r="F25" s="2"/>
+      <c r="G25" s="2"/>
+      <c r="H25" s="2"/>
+      <c r="I25" s="2"/>
+      <c r="J25" s="2"/>
+      <c r="K25" s="2"/>
+      <c r="L25" s="2"/>
       <c r="M25" s="2" t="s">
-        <v>225</v>
+        <v>336</v>
       </c>
       <c r="N25" s="2" t="s">
-        <v>226</v>
+        <v>337</v>
       </c>
     </row>
     <row r="26" spans="1:14" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="E26" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="G26" s="2" t="s">
-        <v>237</v>
-      </c>
-      <c r="H26" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="I26" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="J26" s="2" t="s">
-        <v>204</v>
-      </c>
-      <c r="K26" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="L26" s="2" t="s">
-        <v>214</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>365</v>
+      </c>
+      <c r="C26" s="2"/>
+      <c r="D26" s="2"/>
+      <c r="E26" s="2"/>
+      <c r="F26" s="2"/>
+      <c r="G26" s="2"/>
+      <c r="H26" s="2"/>
+      <c r="I26" s="2"/>
+      <c r="J26" s="2"/>
+      <c r="K26" s="2"/>
+      <c r="L26" s="2"/>
       <c r="M26" s="2" t="s">
-        <v>223</v>
+        <v>338</v>
       </c>
       <c r="N26" s="2" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="27" spans="1:14" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="E27" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="F27" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="G27" s="2"/>
-      <c r="H27" s="2"/>
-      <c r="I27" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="J27" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="K27" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="L27" s="2" t="s">
-        <v>216</v>
-      </c>
-      <c r="M27" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="N27" s="2" t="s">
-        <v>192</v>
-      </c>
+        <v>339</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A27" s="3"/>
+      <c r="B27" s="3"/>
+      <c r="C27" s="3"/>
+      <c r="D27" s="3"/>
+      <c r="E27" s="3"/>
+      <c r="F27" s="3"/>
+      <c r="G27" s="3"/>
+      <c r="H27" s="3"/>
+      <c r="I27" s="3"/>
+      <c r="J27" s="3"/>
+      <c r="K27" s="3"/>
+      <c r="L27" s="3"/>
+      <c r="M27" s="3"/>
+      <c r="N27" s="3"/>
     </row>
     <row r="28" spans="1:14" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>15</v>
+        <v>12</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>366</v>
       </c>
       <c r="C28" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="H28" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="D28" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="E28" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="F28" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="G28" s="2"/>
-      <c r="H28" s="2"/>
       <c r="I28" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="J28" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="K28" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="L28" s="2" t="s">
         <v>205</v>
       </c>
-      <c r="J28" s="2" t="s">
+      <c r="M28" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="N28" s="2" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="A29" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>366</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="H29" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="I29" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="J29" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="K29" s="2" t="s">
         <v>206</v>
       </c>
-      <c r="K28" s="2" t="s">
+      <c r="L29" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="M29" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="N29" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="L28" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="M28" s="2"/>
-      <c r="N28" s="2"/>
-    </row>
-    <row r="29" spans="1:14" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>292</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>293</v>
-      </c>
-      <c r="E29" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="F29" s="2" t="s">
-        <v>181</v>
-      </c>
-      <c r="G29" s="2"/>
-      <c r="H29" s="2"/>
-      <c r="I29" s="2" t="s">
-        <v>311</v>
-      </c>
-      <c r="J29" s="2" t="s">
-        <v>312</v>
-      </c>
-      <c r="K29" s="2" t="s">
-        <v>240</v>
-      </c>
-      <c r="L29" s="2" t="s">
-        <v>241</v>
-      </c>
-      <c r="M29" s="2"/>
-      <c r="N29" s="2"/>
     </row>
     <row r="30" spans="1:14" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
+        <v>12</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>366</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>168</v>
+      </c>
       <c r="E30" s="2" t="s">
-        <v>182</v>
+        <v>42</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="G30" s="2"/>
-      <c r="H30" s="2"/>
-      <c r="I30" s="2"/>
-      <c r="J30" s="2"/>
+        <v>43</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="I30" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="J30" s="2" t="s">
+        <v>102</v>
+      </c>
       <c r="K30" s="2" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="L30" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M30" s="2"/>
-      <c r="N30" s="2"/>
-    </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A31" s="3"/>
-      <c r="B31" s="3"/>
-      <c r="C31" s="3"/>
-      <c r="D31" s="3"/>
-      <c r="E31" s="3"/>
-      <c r="F31" s="3"/>
-      <c r="G31" s="3"/>
-      <c r="H31" s="3"/>
-      <c r="I31" s="3"/>
-      <c r="J31" s="3"/>
-      <c r="K31" s="3"/>
-      <c r="L31" s="3"/>
-      <c r="M31" s="3"/>
-      <c r="N31" s="3"/>
+        <v>19</v>
+      </c>
+      <c r="M30" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="N30" s="2" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>366</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="H31" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="I31" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="J31" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="K31" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="L31" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="M31" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="N31" s="2" t="s">
+        <v>219</v>
+      </c>
     </row>
     <row r="32" spans="1:14" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>17</v>
+        <v>12</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>366</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>227</v>
+        <v>165</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>228</v>
+        <v>166</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>248</v>
+        <v>171</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>249</v>
-      </c>
-      <c r="G32" s="2" t="s">
-        <v>275</v>
-      </c>
-      <c r="H32" s="2" t="s">
-        <v>276</v>
-      </c>
-      <c r="I32" s="4" t="s">
-        <v>319</v>
-      </c>
-      <c r="J32" s="4" t="s">
-        <v>320</v>
+        <v>172</v>
+      </c>
+      <c r="G32" s="2"/>
+      <c r="H32" s="2"/>
+      <c r="I32" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="J32" s="2" t="s">
+        <v>203</v>
       </c>
       <c r="K32" s="2" t="s">
-        <v>281</v>
+        <v>210</v>
       </c>
       <c r="L32" s="2" t="s">
-        <v>282</v>
+        <v>211</v>
       </c>
       <c r="M32" s="2" t="s">
-        <v>60</v>
+        <v>186</v>
       </c>
       <c r="N32" s="2" t="s">
-        <v>61</v>
+        <v>187</v>
       </c>
     </row>
     <row r="33" spans="1:14" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>17</v>
+        <v>12</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>366</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>229</v>
+        <v>179</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>230</v>
+        <v>180</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>250</v>
+        <v>173</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>251</v>
-      </c>
-      <c r="G33" s="2" t="s">
-        <v>258</v>
-      </c>
-      <c r="H33" s="2" t="s">
-        <v>259</v>
-      </c>
+        <v>174</v>
+      </c>
+      <c r="G33" s="2"/>
+      <c r="H33" s="2"/>
       <c r="I33" s="2" t="s">
-        <v>268</v>
+        <v>200</v>
       </c>
       <c r="J33" s="2" t="s">
-        <v>269</v>
+        <v>201</v>
       </c>
       <c r="K33" s="2" t="s">
-        <v>283</v>
+        <v>212</v>
       </c>
       <c r="L33" s="2" t="s">
-        <v>284</v>
+        <v>213</v>
       </c>
       <c r="M33" s="2" t="s">
-        <v>294</v>
+        <v>340</v>
       </c>
       <c r="N33" s="2" t="s">
-        <v>295</v>
+        <v>341</v>
       </c>
     </row>
     <row r="34" spans="1:14" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>17</v>
+        <v>12</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>366</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>231</v>
+        <v>287</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>232</v>
+        <v>288</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>252</v>
+        <v>175</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="G34" s="2" t="s">
-        <v>260</v>
-      </c>
-      <c r="H34" s="2" t="s">
-        <v>261</v>
-      </c>
+        <v>176</v>
+      </c>
+      <c r="G34" s="2"/>
+      <c r="H34" s="2"/>
       <c r="I34" s="2" t="s">
-        <v>270</v>
+        <v>306</v>
       </c>
       <c r="J34" s="2" t="s">
-        <v>128</v>
+        <v>307</v>
       </c>
       <c r="K34" s="2" t="s">
-        <v>285</v>
+        <v>235</v>
       </c>
       <c r="L34" s="2" t="s">
-        <v>286</v>
-      </c>
-      <c r="M34" s="2"/>
-      <c r="N34" s="2"/>
+        <v>236</v>
+      </c>
+      <c r="M34" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="N34" s="2" t="s">
+        <v>343</v>
+      </c>
     </row>
     <row r="35" spans="1:14" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B35" s="2" t="s">
-        <v>17</v>
+        <v>12</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>366</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>233</v>
+        <v>177</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="E35" s="2" t="s">
-        <v>254</v>
-      </c>
-      <c r="F35" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="G35" s="2" t="s">
-        <v>262</v>
-      </c>
-      <c r="H35" s="2" t="s">
-        <v>263</v>
-      </c>
-      <c r="I35" s="2" t="s">
-        <v>271</v>
-      </c>
-      <c r="J35" s="2" t="s">
-        <v>272</v>
-      </c>
+        <v>178</v>
+      </c>
+      <c r="E35" s="2"/>
+      <c r="F35" s="2"/>
+      <c r="G35" s="2"/>
+      <c r="H35" s="2"/>
+      <c r="I35" s="2"/>
+      <c r="J35" s="2"/>
       <c r="K35" s="2" t="s">
-        <v>287</v>
+        <v>20</v>
       </c>
       <c r="L35" s="2" t="s">
-        <v>288</v>
+        <v>21</v>
       </c>
       <c r="M35" s="2"/>
       <c r="N35" s="2"/>
     </row>
     <row r="36" spans="1:14" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B36" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>235</v>
-      </c>
-      <c r="D36" s="2" t="s">
-        <v>236</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>366</v>
+      </c>
+      <c r="C36" s="2"/>
+      <c r="D36" s="2"/>
       <c r="E36" s="2"/>
       <c r="F36" s="2"/>
-      <c r="G36" s="2" t="s">
-        <v>264</v>
-      </c>
-      <c r="H36" s="2" t="s">
-        <v>265</v>
-      </c>
-      <c r="I36" s="2" t="s">
-        <v>277</v>
-      </c>
-      <c r="J36" s="2" t="s">
-        <v>278</v>
-      </c>
+      <c r="G36" s="2"/>
+      <c r="H36" s="2"/>
+      <c r="I36" s="2"/>
+      <c r="J36" s="2"/>
       <c r="K36" s="2" t="s">
-        <v>289</v>
+        <v>344</v>
       </c>
       <c r="L36" s="2" t="s">
-        <v>267</v>
+        <v>345</v>
       </c>
       <c r="M36" s="2"/>
       <c r="N36" s="2"/>
     </row>
     <row r="37" spans="1:14" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B37" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>244</v>
-      </c>
-      <c r="D37" s="2" t="s">
-        <v>245</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="B37" s="5" t="s">
+        <v>366</v>
+      </c>
+      <c r="C37" s="2"/>
+      <c r="D37" s="2"/>
       <c r="E37" s="2"/>
       <c r="F37" s="2"/>
-      <c r="G37" s="2" t="s">
-        <v>296</v>
-      </c>
-      <c r="H37" s="2" t="s">
-        <v>297</v>
-      </c>
-      <c r="I37" s="2" t="s">
-        <v>256</v>
-      </c>
-      <c r="J37" s="2" t="s">
-        <v>257</v>
-      </c>
+      <c r="G37" s="2"/>
+      <c r="H37" s="2"/>
+      <c r="I37" s="2"/>
+      <c r="J37" s="2"/>
       <c r="K37" s="2" t="s">
-        <v>266</v>
+        <v>346</v>
       </c>
       <c r="L37" s="2" t="s">
-        <v>267</v>
+        <v>347</v>
       </c>
       <c r="M37" s="2"/>
       <c r="N37" s="2"/>
     </row>
     <row r="38" spans="1:14" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B38" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>239</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="B38" s="5" t="s">
+        <v>366</v>
+      </c>
+      <c r="C38" s="2"/>
+      <c r="D38" s="2"/>
       <c r="E38" s="2"/>
       <c r="F38" s="2"/>
-      <c r="G38" s="2" t="s">
-        <v>298</v>
-      </c>
-      <c r="H38" s="2" t="s">
-        <v>299</v>
-      </c>
+      <c r="G38" s="2"/>
+      <c r="H38" s="2"/>
       <c r="I38" s="2"/>
       <c r="J38" s="2"/>
       <c r="K38" s="2" t="s">
-        <v>139</v>
+        <v>348</v>
       </c>
       <c r="L38" s="2" t="s">
-        <v>33</v>
+        <v>349</v>
       </c>
       <c r="M38" s="2"/>
       <c r="N38" s="2"/>
     </row>
     <row r="39" spans="1:14" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C39" s="2" t="s">
-        <v>313</v>
-      </c>
-      <c r="D39" s="2" t="s">
-        <v>314</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="B39" s="5" t="s">
+        <v>366</v>
+      </c>
+      <c r="C39" s="2"/>
+      <c r="D39" s="2"/>
       <c r="E39" s="2"/>
       <c r="F39" s="2"/>
-      <c r="G39" s="2" t="s">
-        <v>300</v>
-      </c>
-      <c r="H39" s="2" t="s">
-        <v>301</v>
-      </c>
+      <c r="G39" s="2"/>
+      <c r="H39" s="2"/>
       <c r="I39" s="2"/>
       <c r="J39" s="2"/>
       <c r="K39" s="2" t="s">
-        <v>305</v>
+        <v>350</v>
       </c>
       <c r="L39" s="2" t="s">
-        <v>306</v>
+        <v>351</v>
       </c>
       <c r="M39" s="2"/>
       <c r="N39" s="2"/>
     </row>
-    <row r="40" spans="1:14" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C40" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="E40" s="2"/>
-      <c r="F40" s="2"/>
-      <c r="G40" s="2" t="s">
+    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A40" s="3"/>
+      <c r="B40" s="3"/>
+      <c r="C40" s="3"/>
+      <c r="D40" s="3"/>
+      <c r="E40" s="3"/>
+      <c r="F40" s="3"/>
+      <c r="G40" s="3"/>
+      <c r="H40" s="3"/>
+      <c r="I40" s="3"/>
+      <c r="J40" s="3"/>
+      <c r="K40" s="3"/>
+      <c r="L40" s="3"/>
+      <c r="M40" s="3"/>
+      <c r="N40" s="3"/>
+    </row>
+    <row r="41" spans="1:14" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A41" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B41" s="5" t="s">
+        <v>367</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="H41" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="I41" s="4" t="s">
+        <v>314</v>
+      </c>
+      <c r="J41" s="4" t="s">
+        <v>315</v>
+      </c>
+      <c r="K41" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="L41" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="M41" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="N41" s="2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A42" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B42" s="5" t="s">
+        <v>367</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="H42" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="I42" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="J42" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="K42" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="L42" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="M42" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="N42" s="2" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A43" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B43" s="5" t="s">
+        <v>367</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="G43" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="H43" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="I43" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="J43" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="K43" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="L43" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="M43" s="2" t="s">
+        <v>356</v>
+      </c>
+      <c r="N43" s="2" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A44" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B44" s="5" t="s">
+        <v>367</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="G44" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="H44" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="I44" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="J44" s="2" t="s">
         <v>273</v>
       </c>
-      <c r="H40" s="2" t="s">
-        <v>274</v>
-      </c>
-      <c r="I40" s="2"/>
-      <c r="J40" s="2"/>
-      <c r="K40" s="2" t="s">
-        <v>307</v>
-      </c>
-      <c r="L40" s="2" t="s">
+      <c r="K44" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="L44" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="M44" s="2" t="s">
+        <v>358</v>
+      </c>
+      <c r="N44" s="2" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="45" spans="1:14" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="A45" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B45" s="5" t="s">
+        <v>367</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="E45" s="2"/>
+      <c r="F45" s="2"/>
+      <c r="G45" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="H45" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="I45" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="J45" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="K45" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="L45" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="M45" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="N45" s="2" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="46" spans="1:14" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="A46" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B46" s="5" t="s">
+        <v>367</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="E46" s="2"/>
+      <c r="F46" s="2"/>
+      <c r="G46" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="H46" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="I46" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="J46" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="K46" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="L46" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="M46" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="N46" s="2" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="47" spans="1:14" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A47" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B47" s="5" t="s">
+        <v>367</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="E47" s="2"/>
+      <c r="F47" s="2"/>
+      <c r="G47" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="H47" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="I47" s="2" t="s">
+        <v>354</v>
+      </c>
+      <c r="J47" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="K47" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="L47" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="M47" s="2"/>
+      <c r="N47" s="2"/>
+    </row>
+    <row r="48" spans="1:14" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A48" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B48" s="5" t="s">
+        <v>367</v>
+      </c>
+      <c r="C48" s="2" t="s">
         <v>308</v>
       </c>
-      <c r="M40" s="2"/>
-      <c r="N40" s="2"/>
-    </row>
-    <row r="41" spans="1:14" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C41" s="2"/>
-      <c r="D41" s="2"/>
-      <c r="E41" s="2"/>
-      <c r="F41" s="2"/>
-      <c r="G41" s="2" t="s">
-        <v>242</v>
-      </c>
-      <c r="H41" s="2" t="s">
-        <v>243</v>
-      </c>
-      <c r="I41" s="2"/>
-      <c r="J41" s="2"/>
-      <c r="K41" s="2" t="s">
+      <c r="D48" s="2" t="s">
         <v>309</v>
       </c>
-      <c r="L41" s="2" t="s">
-        <v>310</v>
-      </c>
-      <c r="M41" s="2"/>
-      <c r="N41" s="2"/>
-    </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A42" s="3"/>
-      <c r="B42" s="3"/>
-      <c r="C42" s="3"/>
-      <c r="D42" s="3"/>
-      <c r="E42" s="3"/>
-      <c r="F42" s="3"/>
-      <c r="G42" s="3"/>
-      <c r="H42" s="3"/>
-      <c r="I42" s="3"/>
-      <c r="J42" s="3"/>
-      <c r="K42" s="3"/>
-      <c r="L42" s="3"/>
-      <c r="M42" s="3"/>
-      <c r="N42" s="3"/>
+      <c r="E48" s="2"/>
+      <c r="F48" s="2"/>
+      <c r="G48" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="H48" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="I48" s="2"/>
+      <c r="J48" s="2"/>
+      <c r="K48" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="L48" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="M48" s="2"/>
+      <c r="N48" s="2"/>
+    </row>
+    <row r="49" spans="1:14" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A49" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B49" s="5" t="s">
+        <v>367</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="E49" s="2"/>
+      <c r="F49" s="2"/>
+      <c r="G49" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="H49" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="I49" s="2"/>
+      <c r="J49" s="2"/>
+      <c r="K49" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="L49" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="M49" s="2"/>
+      <c r="N49" s="2"/>
+    </row>
+    <row r="50" spans="1:14" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A50" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B50" s="5" t="s">
+        <v>367</v>
+      </c>
+      <c r="C50" s="2"/>
+      <c r="D50" s="2"/>
+      <c r="E50" s="2"/>
+      <c r="F50" s="2"/>
+      <c r="G50" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="H50" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="I50" s="2"/>
+      <c r="J50" s="2"/>
+      <c r="K50" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="L50" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="M50" s="2"/>
+      <c r="N50" s="2"/>
+    </row>
+    <row r="51" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A51" s="3"/>
+      <c r="B51" s="3"/>
+      <c r="C51" s="3"/>
+      <c r="D51" s="3"/>
+      <c r="E51" s="3"/>
+      <c r="F51" s="3"/>
+      <c r="G51" s="3"/>
+      <c r="H51" s="3"/>
+      <c r="I51" s="3"/>
+      <c r="J51" s="3"/>
+      <c r="K51" s="3"/>
+      <c r="L51" s="3"/>
+      <c r="M51" s="3"/>
+      <c r="N51" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>